<commit_message>
feat: integrate sample groups into modeling dataset
</commit_message>
<xml_diff>
--- a/tests/fixtures/metadata.xlsx
+++ b/tests/fixtures/metadata.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,6 +439,16 @@
           <t>type</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nr</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -451,6 +461,16 @@
           <t>other</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -463,6 +483,16 @@
           <t>cocaine</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -471,6 +501,16 @@
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -481,6 +521,16 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>cocaine</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>

</xml_diff>